<commit_message>
Wstępny schemat oraz projekt PCB
</commit_message>
<xml_diff>
--- a/Kosztorys.xlsx
+++ b/Kosztorys.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="102">
   <si>
     <t xml:space="preserve">UKŁADY SCALONE</t>
   </si>
@@ -46,10 +46,10 @@
     <t xml:space="preserve">Klasa</t>
   </si>
   <si>
-    <t xml:space="preserve">konwerter logiczny</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TXS0102DCUR</t>
+    <t xml:space="preserve">transciver CAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP2562-E/SN</t>
   </si>
   <si>
     <t xml:space="preserve">TME</t>
@@ -58,36 +58,30 @@
     <t xml:space="preserve">Industrial</t>
   </si>
   <si>
-    <t xml:space="preserve">transceiver CAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TJA1050T/CM</t>
+    <t xml:space="preserve">potencjometr cyfrowy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCP4661-103E/ST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wzmacniacz operacyjny</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NCV21872DMR2G </t>
   </si>
   <si>
     <t xml:space="preserve">Automotive</t>
   </si>
   <si>
-    <t xml:space="preserve">potencjometr cyfrowy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCP4661-103E/ST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wzmacniacz operacyjny</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NCV21872DMR2G </t>
+    <t xml:space="preserve">microkontroler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STM32F105RBT6</t>
   </si>
   <si>
     <t xml:space="preserve">SUMA</t>
   </si>
   <si>
-    <t xml:space="preserve">microkontroler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STM32F105RBT6</t>
-  </si>
-  <si>
     <t xml:space="preserve">LDO 3.3V</t>
   </si>
   <si>
@@ -133,6 +127,9 @@
     <t xml:space="preserve">43045-0621</t>
   </si>
   <si>
+    <t xml:space="preserve">*</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gniazdo Micro-Fit 3.0 4pin</t>
   </si>
   <si>
@@ -143,6 +140,165 @@
   </si>
   <si>
     <t xml:space="preserve">43045-0800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gniazdo USB C 16 pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB4105-GF-A-120 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gniazdo DC Jack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC-GK2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DROBNICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bezpiecznik polimerowy 500mA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0ZCJ0050FF2G </t>
+  </si>
+  <si>
+    <t xml:space="preserve">bezpiecznik polimerowy 1.25A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1812L125/16DR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kwarc 25MHz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3225-25M-SR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mikroprzełącznik TACT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PTS645SK43SMTR92 LFS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED zielona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSG80603C1E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED pomaranczowa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSO50603C1E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kondensator 10nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C0805C103K1RACTU </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kondensator 100nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08055C104JAT2A </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kondensator 10uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM21BR60J106KE19L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kondensator 1nF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KGM21NR71H102KT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kondensator 10pF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08055A100JAT2A </t>
+  </si>
+  <si>
+    <t xml:space="preserve">dioda shottky 2A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezystor 100R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRCW0805100RFKTABC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezystor 1k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRCW08051K00FKTABC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">22R 1206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRCW120622R0FKTABC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1k 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-075K1L </t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.1k 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-079K1L </t>
+  </si>
+  <si>
+    <t xml:space="preserve">22R 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-0722RL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">120R 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WR08X1200FTL </t>
+  </si>
+  <si>
+    <t xml:space="preserve">270R 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRCW0805270RFKTABC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRCW080510K0FKEA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">22k 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRCW080522K0FKEA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">82k 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ERA6AEB823V </t>
+  </si>
+  <si>
+    <t xml:space="preserve">33k 0805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-0733KL </t>
   </si>
   <si>
     <t xml:space="preserve">NARZĘDZIA</t>
@@ -180,7 +336,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -217,6 +373,12 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="238"/>
     </font>
     <font>
       <sz val="10"/>
@@ -268,7 +430,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -305,16 +467,20 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -440,7 +606,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.16"/>
@@ -479,7 +645,7 @@
       <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -497,13 +663,13 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1.93</v>
+        <v>4.23</v>
       </c>
       <c r="F3" s="5" t="n">
         <f aca="false">PRODUCT(D3,E3)*1.23</f>
-        <v>2.3739</v>
-      </c>
-      <c r="G3" s="0" t="s">
+        <v>5.2029</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -521,22 +687,22 @@
         <v>1</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>3.78</v>
+        <v>5.34</v>
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">PRODUCT(D4,E4)*1.23</f>
-        <v>4.6494</v>
-      </c>
-      <c r="G4" s="0" t="s">
-        <v>14</v>
+        <v>6.5682</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>10</v>
@@ -545,14 +711,14 @@
         <v>1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>5.34</v>
-      </c>
-      <c r="F5" s="5" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="F5" s="6" t="n">
         <f aca="false">PRODUCT(D5,E5)*1.23</f>
-        <v>6.5682</v>
-      </c>
-      <c r="G5" s="0" t="s">
-        <v>11</v>
+        <v>2.9643</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -565,28 +731,28 @@
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>2.41</v>
+        <v>25.31</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">PRODUCT(D6,E6)*1.23</f>
-        <v>2.9643</v>
-      </c>
-      <c r="G6" s="0" t="s">
-        <v>14</v>
+        <v>31.1313</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -595,88 +761,64 @@
       <c r="D7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="3" t="n">
-        <v>25.31</v>
+      <c r="E7" s="5" t="n">
+        <v>1.926</v>
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">PRODUCT(D7,E7)*1.23</f>
-        <v>31.1313</v>
-      </c>
-      <c r="G7" s="0" t="s">
-        <v>11</v>
+        <v>2.36898</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="I7" s="5" t="n">
-        <f aca="false">SUM(F3:F33)</f>
-        <v>197.25098</v>
+        <f aca="false">SUM(F3:F70)</f>
+        <v>300.3363575</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>1.926</v>
+      <c r="E8" s="3" t="n">
+        <v>1.48</v>
       </c>
       <c r="F8" s="6" t="n">
         <f aca="false">PRODUCT(D8,E8)*1.23</f>
-        <v>2.36898</v>
-      </c>
-      <c r="G8" s="0" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+        <v>1.8204</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <f aca="false">PRODUCT(D9,E9)*1.23</f>
-        <v>1.8204</v>
-      </c>
-      <c r="G9" s="0" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11" t="n">
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9" t="n">
         <f aca="false">PRODUCT(D12,E12)*1.23</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>10</v>
@@ -691,16 +833,16 @@
         <f aca="false">PRODUCT(D13,E13)*1.23</f>
         <v>2.0541</v>
       </c>
-      <c r="G13" s="0" t="s">
-        <v>14</v>
+      <c r="G13" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>10</v>
@@ -715,16 +857,16 @@
         <f aca="false">PRODUCT(D14,E14)*1.23</f>
         <v>2.6814</v>
       </c>
-      <c r="G14" s="0" t="s">
-        <v>14</v>
+      <c r="G14" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>10</v>
@@ -739,40 +881,40 @@
         <f aca="false">PRODUCT(D15,E15)*1.23</f>
         <v>1.353</v>
       </c>
-      <c r="G15" s="0" t="s">
-        <v>14</v>
+      <c r="G15" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>0.382</v>
       </c>
       <c r="F16" s="6" t="n">
         <f aca="false">PRODUCT(D16,E16)*1.23</f>
-        <v>14.0958</v>
-      </c>
-      <c r="G16" s="0" t="s">
-        <v>14</v>
+        <v>16.4451</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>10</v>
@@ -787,16 +929,19 @@
         <f aca="false">PRODUCT(D17,E17)*1.23</f>
         <v>7.1832</v>
       </c>
-      <c r="G17" s="0" t="s">
-        <v>14</v>
+      <c r="G17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>10</v>
@@ -811,16 +956,16 @@
         <f aca="false">PRODUCT(D18,E18)*1.23</f>
         <v>4.551</v>
       </c>
-      <c r="G18" s="0" t="s">
-        <v>14</v>
+      <c r="G18" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>39</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>40</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>10</v>
@@ -835,135 +980,695 @@
         <f aca="false">PRODUCT(D19,E19)*1.23</f>
         <v>5.6457</v>
       </c>
-      <c r="G19" s="0" t="s">
-        <v>14</v>
+      <c r="G19" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="6"/>
+      <c r="A20" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <f aca="false">PRODUCT(D20,E20)*1.23</f>
+        <v>3.4317</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11" t="n">
+      <c r="A21" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F21" s="6" t="n">
         <f aca="false">PRODUCT(D21,E21)*1.23</f>
+        <v>5.0553</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2" t="n">
+        <f aca="false">PRODUCT(D23,E23)*1.23</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="7" t="n">
-        <v>22.61</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <f aca="false">PRODUCT(D22,E22)*1.23</f>
-        <v>27.8103</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-    </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
+      <c r="A24" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <f aca="false">PRODUCT(D24,E24)*1.23</f>
+        <v>5.1045</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="D25" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <f aca="false">PRODUCT(D25,E25)*1.23</f>
+        <v>3.8376</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>1.205</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <f aca="false">PRODUCT(D26,E26)*1.23</f>
+        <v>5.9286</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>1.256</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <f aca="false">PRODUCT(D27,E27)*1.23</f>
+        <v>6.17952</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>0.3296</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <f aca="false">PRODUCT(D28,E28)*1.23</f>
+        <v>4.05408</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="E25" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F25" s="7" t="n">
+      <c r="E29" s="5" t="n">
+        <v>0.6757</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <f aca="false">PRODUCT(D29,E29)*1.23</f>
+        <v>4.155555</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="3" t="n">
         <v>50</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="11"/>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D28" s="7" t="n">
+      <c r="E30" s="5" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <f aca="false">PRODUCT(D30,E30)*1.23</f>
+        <v>5.1045</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0.0995</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <f aca="false">PRODUCT(D31,E31)*1.23</f>
+        <v>7.3431</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>0.1959</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <f aca="false">PRODUCT(D32,E32)*1.23</f>
+        <v>6.023925</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>0.0767</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <f aca="false">PRODUCT(D33,E33)*1.23</f>
+        <v>4.71705</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>0.1149</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <f aca="false">PRODUCT(D34,E34)*1.23</f>
+        <v>3.533175</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>0.5256</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <f aca="false">PRODUCT(D35,E35)*1.23</f>
+        <v>3.23244</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>0.03957</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <f aca="false">PRODUCT(D36,E36)*1.23</f>
+        <v>2.433555</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>0.01861</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <f aca="false">PRODUCT(D37,E37)*1.23</f>
+        <v>2.28903</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>0.02808</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <f aca="false">PRODUCT(D38,E38)*1.23</f>
+        <v>3.45384</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>0.0609</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <f aca="false">PRODUCT(D39,E39)*1.23</f>
+        <v>3.74535</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>0.04206</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <f aca="false">PRODUCT(D40,E40)*1.23</f>
+        <v>2.58669</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>0.02928</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <f aca="false">PRODUCT(D41,E41)*1.23</f>
+        <v>1.80072</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>0.10465</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <f aca="false">PRODUCT(D42,E42)*1.23</f>
+        <v>3.2179875</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>0.03764</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <f aca="false">PRODUCT(D43,E43)*1.23</f>
+        <v>2.31486</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>0.0298</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <f aca="false">PRODUCT(D44,E44)*1.23</f>
+        <v>1.8327</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>0.0725</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <f aca="false">PRODUCT(D45,E45)*1.23</f>
+        <v>2.229375</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>0.2568</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <f aca="false">PRODUCT(D46,E46)*1.23</f>
+        <v>6.31728</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>0.04283</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <f aca="false">PRODUCT(D47,E47)*1.23</f>
+        <v>2.634045</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9" t="n">
+        <f aca="false">PRODUCT(D48,E48)*1.23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B49" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="7" t="n">
+      <c r="E49" s="7" t="n">
+        <v>22.61</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <f aca="false">PRODUCT(D49,E49)*1.23</f>
+        <v>27.8103</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B51" s="9"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="9"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B54" s="9"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="F28" s="7" t="n">
+      <c r="F55" s="7" t="n">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A54:F54"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="TME"/>
@@ -972,16 +1677,41 @@
     <hyperlink ref="C6" r:id="rId4" display="TME"/>
     <hyperlink ref="C7" r:id="rId5" display="TME"/>
     <hyperlink ref="C8" r:id="rId6" display="TME"/>
-    <hyperlink ref="C9" r:id="rId7" display="TME"/>
-    <hyperlink ref="C13" r:id="rId8" display="TME"/>
-    <hyperlink ref="C14" r:id="rId9" display="TME"/>
-    <hyperlink ref="C15" r:id="rId10" display="TME"/>
-    <hyperlink ref="C16" r:id="rId11" display="TME"/>
-    <hyperlink ref="C17" r:id="rId12" display="TME"/>
-    <hyperlink ref="C18" r:id="rId13" display="TME"/>
-    <hyperlink ref="C19" r:id="rId14" display="TME"/>
-    <hyperlink ref="C22" r:id="rId15" display="TME"/>
-    <hyperlink ref="C25" r:id="rId16" display="Allegro"/>
+    <hyperlink ref="C13" r:id="rId7" display="TME"/>
+    <hyperlink ref="C14" r:id="rId8" display="TME"/>
+    <hyperlink ref="C15" r:id="rId9" display="TME"/>
+    <hyperlink ref="C16" r:id="rId10" display="TME"/>
+    <hyperlink ref="C17" r:id="rId11" display="TME"/>
+    <hyperlink ref="C18" r:id="rId12" display="TME"/>
+    <hyperlink ref="C19" r:id="rId13" display="TME"/>
+    <hyperlink ref="C20" r:id="rId14" display="TME"/>
+    <hyperlink ref="C21" r:id="rId15" display="TME"/>
+    <hyperlink ref="C24" r:id="rId16" display="TME"/>
+    <hyperlink ref="C25" r:id="rId17" display="TME"/>
+    <hyperlink ref="C26" r:id="rId18" display="TME"/>
+    <hyperlink ref="C27" r:id="rId19" display="TME"/>
+    <hyperlink ref="C28" r:id="rId20" display="TME"/>
+    <hyperlink ref="C29" r:id="rId21" display="TME"/>
+    <hyperlink ref="C30" r:id="rId22" display="TME"/>
+    <hyperlink ref="C31" r:id="rId23" display="TME"/>
+    <hyperlink ref="C32" r:id="rId24" display="TME"/>
+    <hyperlink ref="C33" r:id="rId25" display="TME"/>
+    <hyperlink ref="C34" r:id="rId26" display="TME"/>
+    <hyperlink ref="C35" r:id="rId27" display="TME"/>
+    <hyperlink ref="C36" r:id="rId28" display="TME"/>
+    <hyperlink ref="C37" r:id="rId29" display="TME"/>
+    <hyperlink ref="C38" r:id="rId30" display="TME"/>
+    <hyperlink ref="C39" r:id="rId31" display="TME"/>
+    <hyperlink ref="C40" r:id="rId32" display="TME"/>
+    <hyperlink ref="C41" r:id="rId33" display="TME"/>
+    <hyperlink ref="C42" r:id="rId34" display="TME"/>
+    <hyperlink ref="C43" r:id="rId35" display="TME"/>
+    <hyperlink ref="C44" r:id="rId36" display="TME"/>
+    <hyperlink ref="C45" r:id="rId37" display="TME"/>
+    <hyperlink ref="C46" r:id="rId38" display="TME"/>
+    <hyperlink ref="C47" r:id="rId39" display="TME"/>
+    <hyperlink ref="C49" r:id="rId40" display="TME"/>
+    <hyperlink ref="C52" r:id="rId41" display="Allegro"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
Wykonano finalne PCB dla forZero_1v0
</commit_message>
<xml_diff>
--- a/Kosztorys.xlsx
+++ b/Kosztorys.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="105">
   <si>
     <t xml:space="preserve">UKŁADY SCALONE</t>
   </si>
@@ -58,6 +58,9 @@
     <t xml:space="preserve">Industrial</t>
   </si>
   <si>
+    <t xml:space="preserve">*</t>
+  </si>
+  <si>
     <t xml:space="preserve">potencjometr cyfrowy</t>
   </si>
   <si>
@@ -127,9 +130,6 @@
     <t xml:space="preserve">43045-0621</t>
   </si>
   <si>
-    <t xml:space="preserve">*</t>
-  </si>
-  <si>
     <t xml:space="preserve">Gniazdo Micro-Fit 3.0 4pin</t>
   </si>
   <si>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Gniazdo DC Jack</t>
   </si>
   <si>
-    <t xml:space="preserve">PC-GK2.1</t>
+    <t xml:space="preserve">DC-10A FC68148 </t>
   </si>
   <si>
     <t xml:space="preserve">DROBNICA</t>
@@ -202,7 +202,7 @@
     <t xml:space="preserve">kondensator 100nF</t>
   </si>
   <si>
-    <t xml:space="preserve">08055C104JAT2A </t>
+    <t xml:space="preserve">KGM21NR71H104KT </t>
   </si>
   <si>
     <t xml:space="preserve">kondensator 10uF</t>
@@ -307,13 +307,16 @@
     <t xml:space="preserve">AO3400A</t>
   </si>
   <si>
+    <t xml:space="preserve">SUMA TME</t>
+  </si>
+  <si>
     <t xml:space="preserve">NARZĘDZIA</t>
   </si>
   <si>
     <t xml:space="preserve">Topnik w żelu</t>
   </si>
   <si>
-    <t xml:space="preserve">BTFO-81-1</t>
+    <t xml:space="preserve">ART.AGT-179 </t>
   </si>
   <si>
     <t xml:space="preserve">PRZEWODY</t>
@@ -342,7 +345,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -384,13 +387,6 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <charset val="238"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="2"/>
       <charset val="238"/>
     </font>
   </fonts>
@@ -477,19 +473,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -673,22 +669,25 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4.23</v>
+        <v>4.26</v>
       </c>
       <c r="F3" s="5" t="n">
         <f aca="false">PRODUCT(D3,E3)*1.23</f>
-        <v>5.2029</v>
+        <v>5.2398</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="H3" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>10</v>
@@ -706,13 +705,16 @@
       <c r="G4" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="H4" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>10</v>
@@ -728,15 +730,18 @@
         <v>2.9643</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>10</v>
@@ -754,16 +759,19 @@
       <c r="G6" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="H6" s="0" t="s">
+        <v>12</v>
+      </c>
       <c r="I6" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>10</v>
@@ -779,19 +787,22 @@
         <v>2.36898</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H7" s="0" t="s">
+        <v>12</v>
       </c>
       <c r="I7" s="5" t="n">
         <f aca="false">SUM(F3:F70)</f>
-        <v>310.7759825</v>
+        <v>317.190863</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>10</v>
@@ -807,12 +818,15 @@
         <v>1.8204</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H8" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -825,10 +839,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>10</v>
@@ -844,15 +858,18 @@
         <v>2.0541</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H13" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>10</v>
@@ -868,15 +885,18 @@
         <v>2.6814</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H14" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>10</v>
@@ -892,15 +912,18 @@
         <v>1.353</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H15" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>10</v>
@@ -916,15 +939,18 @@
         <v>16.4451</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H16" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>10</v>
@@ -940,10 +966,10 @@
         <v>7.1832</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -967,7 +993,10 @@
         <v>4.551</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H18" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -991,7 +1020,10 @@
         <v>5.6457</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="H19" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1014,26 +1046,32 @@
         <f aca="false">PRODUCT(D20,E20)*1.23</f>
         <v>3.4317</v>
       </c>
+      <c r="H20" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="10" t="s">
         <v>43</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>1.37</v>
+        <v>2.97</v>
       </c>
       <c r="F21" s="6" t="n">
         <f aca="false">PRODUCT(D21,E21)*1.23</f>
-        <v>5.0553</v>
+        <v>3.6531</v>
+      </c>
+      <c r="H21" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1077,6 +1115,9 @@
         <f aca="false">PRODUCT(D24,E24)*1.23</f>
         <v>5.1045</v>
       </c>
+      <c r="H24" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
@@ -1098,6 +1139,9 @@
         <f aca="false">PRODUCT(D25,E25)*1.23</f>
         <v>3.8376</v>
       </c>
+      <c r="H25" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
@@ -1110,14 +1154,17 @@
         <v>10</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>1.205</v>
+        <v>0.656</v>
       </c>
       <c r="F26" s="6" t="n">
         <f aca="false">PRODUCT(D26,E26)*1.23</f>
-        <v>5.9286</v>
+        <v>8.0688</v>
+      </c>
+      <c r="H26" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1140,6 +1187,9 @@
         <f aca="false">PRODUCT(D27,E27)*1.23</f>
         <v>6.17952</v>
       </c>
+      <c r="H27" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
@@ -1161,6 +1211,9 @@
         <f aca="false">PRODUCT(D28,E28)*1.23</f>
         <v>4.05408</v>
       </c>
+      <c r="H28" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
@@ -1182,6 +1235,9 @@
         <f aca="false">PRODUCT(D29,E29)*1.23</f>
         <v>4.155555</v>
       </c>
+      <c r="H29" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
@@ -1203,33 +1259,39 @@
         <f aca="false">PRODUCT(D30,E30)*1.23</f>
         <v>5.1045</v>
       </c>
+      <c r="H30" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="10" t="s">
         <v>60</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.0995</v>
+        <v>0.05633</v>
       </c>
       <c r="F31" s="6" t="n">
         <f aca="false">PRODUCT(D31,E31)*1.23</f>
-        <v>7.3431</v>
+        <v>6.92859</v>
+      </c>
+      <c r="H31" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="11" t="s">
         <v>62</v>
       </c>
       <c r="C32" s="4" t="s">
@@ -1245,6 +1307,9 @@
         <f aca="false">PRODUCT(D32,E32)*1.23</f>
         <v>6.023925</v>
       </c>
+      <c r="H32" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
@@ -1266,12 +1331,15 @@
         <f aca="false">PRODUCT(D33,E33)*1.23</f>
         <v>4.71705</v>
       </c>
+      <c r="H33" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="10" t="s">
         <v>66</v>
       </c>
       <c r="C34" s="4" t="s">
@@ -1287,6 +1355,9 @@
         <f aca="false">PRODUCT(D34,E34)*1.23</f>
         <v>3.533175</v>
       </c>
+      <c r="H34" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
@@ -1308,12 +1379,15 @@
         <f aca="false">PRODUCT(D35,E35)*1.23</f>
         <v>3.23244</v>
       </c>
+      <c r="H35" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="10" t="s">
         <v>70</v>
       </c>
       <c r="C36" s="4" t="s">
@@ -1329,12 +1403,15 @@
         <f aca="false">PRODUCT(D36,E36)*1.23</f>
         <v>2.433555</v>
       </c>
+      <c r="H36" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="10" t="s">
         <v>72</v>
       </c>
       <c r="C37" s="4" t="s">
@@ -1350,12 +1427,15 @@
         <f aca="false">PRODUCT(D37,E37)*1.23</f>
         <v>2.28903</v>
       </c>
+      <c r="H37" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="10" t="s">
         <v>74</v>
       </c>
       <c r="C38" s="4" t="s">
@@ -1371,12 +1451,15 @@
         <f aca="false">PRODUCT(D38,E38)*1.23</f>
         <v>3.45384</v>
       </c>
+      <c r="H38" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="10" t="s">
         <v>76</v>
       </c>
       <c r="C39" s="4" t="s">
@@ -1392,33 +1475,39 @@
         <f aca="false">PRODUCT(D39,E39)*1.23</f>
         <v>3.74535</v>
       </c>
+      <c r="H39" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="10" t="s">
         <v>78</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D40" s="7" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>0.04206</v>
+        <v>0.021146</v>
       </c>
       <c r="F40" s="6" t="n">
         <f aca="false">PRODUCT(D40,E40)*1.23</f>
-        <v>2.58669</v>
+        <v>2.600958</v>
+      </c>
+      <c r="H40" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="10" t="s">
         <v>80</v>
       </c>
       <c r="C41" s="4" t="s">
@@ -1434,33 +1523,39 @@
         <f aca="false">PRODUCT(D41,E41)*1.23</f>
         <v>1.80072</v>
       </c>
+      <c r="H41" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="10" t="s">
         <v>82</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D42" s="7" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="E42" s="7" t="n">
-        <v>0.10465</v>
+        <v>0.02597</v>
       </c>
       <c r="F42" s="6" t="n">
         <f aca="false">PRODUCT(D42,E42)*1.23</f>
-        <v>3.2179875</v>
+        <v>3.19431</v>
+      </c>
+      <c r="H42" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="10" t="s">
         <v>84</v>
       </c>
       <c r="C43" s="4" t="s">
@@ -1476,12 +1571,15 @@
         <f aca="false">PRODUCT(D43,E43)*1.23</f>
         <v>2.31486</v>
       </c>
+      <c r="H43" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="10" t="s">
         <v>86</v>
       </c>
       <c r="C44" s="4" t="s">
@@ -1497,12 +1595,15 @@
         <f aca="false">PRODUCT(D44,E44)*1.23</f>
         <v>1.8327</v>
       </c>
+      <c r="H44" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="10" t="s">
         <v>88</v>
       </c>
       <c r="C45" s="4" t="s">
@@ -1518,12 +1619,15 @@
         <f aca="false">PRODUCT(D45,E45)*1.23</f>
         <v>2.229375</v>
       </c>
+      <c r="H45" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="10" t="s">
         <v>90</v>
       </c>
       <c r="C46" s="4" t="s">
@@ -1539,12 +1643,15 @@
         <f aca="false">PRODUCT(D46,E46)*1.23</f>
         <v>6.31728</v>
       </c>
+      <c r="H46" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B47" s="10" t="s">
         <v>92</v>
       </c>
       <c r="C47" s="4" t="s">
@@ -1560,6 +1667,9 @@
         <f aca="false">PRODUCT(D47,E47)*1.23</f>
         <v>2.634045</v>
       </c>
+      <c r="H47" s="0" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
@@ -1580,6 +1690,9 @@
       <c r="F48" s="6" t="n">
         <f aca="false">PRODUCT(D48,E48)*1.23</f>
         <v>10.439625</v>
+      </c>
+      <c r="H48" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1597,10 +1710,17 @@
       <c r="D50" s="12"/>
       <c r="E50" s="12"/>
       <c r="F50" s="12"/>
+      <c r="H50" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="I50" s="0" t="n">
+        <f aca="false">SUM(F3:F52)</f>
+        <v>237.190863</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B51" s="9"/>
       <c r="C51" s="9"/>
@@ -1613,10 +1733,10 @@
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B52" s="7" t="s">
         <v>97</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>98</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>10</v>
@@ -1625,11 +1745,11 @@
         <v>1</v>
       </c>
       <c r="E52" s="7" t="n">
-        <v>22.61</v>
+        <v>27.54</v>
       </c>
       <c r="F52" s="6" t="n">
         <f aca="false">PRODUCT(D52,E52)*1.23</f>
-        <v>27.8103</v>
+        <v>33.8742</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1642,7 +1762,7 @@
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B54" s="9"/>
       <c r="C54" s="9"/>
@@ -1652,13 +1772,13 @@
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D55" s="7" t="n">
         <v>5</v>
@@ -1680,7 +1800,7 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B57" s="9"/>
       <c r="C57" s="9"/>
@@ -1690,13 +1810,13 @@
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D58" s="7" t="n">
         <v>1</v>

</xml_diff>